<commit_message>
Ma222: normal areas practice down to 15 problems, with varied wording for each kind of area
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ma222/data/NormalAreasPractice-Answers.xlsx
+++ b/Ma222/data/NormalAreasPractice-Answers.xlsx
@@ -522,381 +522,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>18</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>19</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>21</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>22</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>23</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>24</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>26</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>27</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>29</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>30</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>31</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>32</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2286000" cy="866775"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1199,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1527,288 +1152,6 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="72" customHeight="1">
-      <c r="A19" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E19" s="5">
-        <f>NORMSDIST(D19)-NORMSDIST(C19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="72" customHeight="1">
-      <c r="A20" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>-2.3</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="E20" s="5">
-        <f>NORMSDIST(D20)-NORMSDIST(C20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="72" customHeight="1">
-      <c r="A21" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>-0.33</v>
-      </c>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="5">
-        <f>NORMSDIST(C21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="72" customHeight="1">
-      <c r="A22" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Right tail</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="5">
-        <f>1.0-NORMSDIST(C22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="72" customHeight="1">
-      <c r="A23" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>-0.9399999999999999</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="E23" s="5">
-        <f>NORMSDIST(D23)-NORMSDIST(C23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="72" customHeight="1">
-      <c r="A24" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Right tail</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="5">
-        <f>1.0-NORMSDIST(C24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="72" customHeight="1">
-      <c r="A25" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>-1.05</v>
-      </c>
-      <c r="E25" s="5">
-        <f>NORMSDIST(D25)-NORMSDIST(C25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="72" customHeight="1">
-      <c r="A26" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Right tail</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>-2.21</v>
-      </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="5">
-        <f>1.0-NORMSDIST(C26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="72" customHeight="1">
-      <c r="A27" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>-1.33</v>
-      </c>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="5">
-        <f>NORMSDIST(C27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="72" customHeight="1">
-      <c r="A28" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="5">
-        <f>NORMSDIST(C28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="72" customHeight="1">
-      <c r="A29" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>-0.72</v>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E29" s="5">
-        <f>NORMSDIST(D29)-NORMSDIST(C29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="72" customHeight="1">
-      <c r="A30" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="5">
-        <f>NORMSDIST(C30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="72" customHeight="1">
-      <c r="A31" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="5">
-        <f>NORMSDIST(C31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="72" customHeight="1">
-      <c r="A32" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Left tail</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>1.86</v>
-      </c>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="5">
-        <f>NORMSDIST(C32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="72" customHeight="1">
-      <c r="A33" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Area between</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="n">
-        <v>-1.15</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E33" s="5">
-        <f>NORMSDIST(D33)-NORMSDIST(C33)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>